<commit_message>
Add DHI marketing contacts and resolve Eddie Haro
Two DHI addresses supplied by the user resolved to Thomas VanBuskirk
(Digital Marketing Manager) and Viky Kalyta (Marketing Coordinator) via
free keyword search, and confirmed DHI uses flast.

That also fixed an earlier miss: the branch sales manager's surname is
"Haro", not "Garza De Haro" as the source list rendered it, which is why
the name lookup failed. His address follows from the confirmed format.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA3eMoHLG5tHsDy3VcGJJG
</commit_message>
<xml_diff>
--- a/mortgage_shortlist.xlsx
+++ b/mortgage_shortlist.xlsx
@@ -8,11 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Shortlist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Still No Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Call First - No Email" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shortlist'!$A$1:$H$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shortlist'!$A$1:$H$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -69,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -79,9 +78,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -455,9 +451,9 @@
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -667,67 +663,71 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>DHI Mortgage Co. Ltd.</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Eddie Garza De Haro</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>branch sales manager</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>no email found</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>eharo@dhimortgage.com</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>predicted (not verified)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>512-502-0545</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>local market leader / branch decision-maker</t>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker | flast confirmed by 2 DHI addresses you supplied</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>DHI Mortgage Co. Ltd.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Shannon O'Reilly</t>
+          <t>Thomas VanBuskirk</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>mortgage lending</t>
+          <t>Digital Marketing Manager</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>shannon.oreilly@jpmchase.com</t>
+          <t>tvanbuskirk@dhimortgage.com</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -737,39 +737,39 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>512-479-1581</t>
+          <t>512-502-0545</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>producer / loan officer</t>
+          <t>local marketing</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>DHI Mortgage Co. Ltd.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Ashlei Bobo</t>
+          <t>Viky Kalyta</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>mortgage lending</t>
+          <t>Marketing Coordinator</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>ashlei.n.bobo@jpmchase.com</t>
+          <t>vkalyta@dhimortgage.com</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -779,39 +779,39 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>512-479-1581</t>
+          <t>512-502-0545</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>producer / loan officer</t>
+          <t>local marketing</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Taylor Morrison Home Funding Inc.</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>April Whitaker</t>
+          <t>Shannon O'Reilly</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Regional president</t>
+          <t>mortgage lending</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>apwhitaker@taylormorrison.com</t>
+          <t>shannon.oreilly@jpmchase.com</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -821,39 +821,39 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>866-379-5390</t>
+          <t>512-479-1581</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Lennar Mortgage</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Joe Crown</t>
+          <t>Ashlei Bobo</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Division manager</t>
+          <t>mortgage lending</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>joecrown@lennarmortgage.com</t>
+          <t>ashlei.n.bobo@jpmchase.com</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -863,39 +863,39 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>512-418-0550</t>
+          <t>512-479-1581</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Lennar Mortgage</t>
+          <t>Taylor Morrison Home Funding Inc.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Trisha Belliveau</t>
+          <t>April Whitaker</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>production manager</t>
+          <t>Regional president</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>trishabelliveau@lennarmortgage.com</t>
+          <t>apwhitaker@taylormorrison.com</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>512-418-0550</t>
+          <t>866-379-5390</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -927,17 +927,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Kyle Simpson</t>
+          <t>Joe Crown</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Austin mortgage</t>
+          <t>Division manager</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>KyleSimpson@lennarmortgage.com</t>
+          <t>joecrown@lennarmortgage.com</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -952,152 +952,152 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Fairway Independent Mortgage Corp. - Round Rock</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Steve Jacobson</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>no email found</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>512-776-1420</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>company exec (local-HQ shop)</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Lennar Mortgage</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Trisha Belliveau</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>production manager</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>trishabelliveau@lennarmortgage.com</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>512-418-0550</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Lennar Mortgage</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Simpson</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Austin mortgage</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>KyleSimpson@lennarmortgage.com</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>512-418-0550</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Fairway Independent Mortgage Corp. - Round Rock</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Drew Carls</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>drew.carls@fairwaymc.com</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>from your list</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Steve Jacobson</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>no email found</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>512-776-1420</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>no title given</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Velocio Mortgage LLC</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Jonathan Seal</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Area sales manager</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>jseal@velociomortgage.com</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>from your list</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>512-314-7301</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>local market leader / branch decision-maker</t>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>company exec (local-HQ shop)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Velocio Mortgage LLC</t>
+          <t>Fairway Independent Mortgage Corp. - Round Rock</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Jerry Villarreal</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>residential mortgage LO (NMLS 1726390)</t>
-        </is>
-      </c>
+          <t>Drew Carls</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>GVgvillarreal@velociomortgage.com</t>
+          <t>drew.carls@fairwaymc.com</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1107,12 +1107,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>512-314-7301</t>
+          <t>512-776-1420</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>producer / loan officer</t>
+          <t>no title given</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Brandon Burkhardt</t>
+          <t>Jonathan Seal</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>residential mortgage LO (NMLS 917247)</t>
+          <t>Area sales manager</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>BBurkhardt@velociomortgage.com</t>
+          <t>jseal@velociomortgage.com</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1154,34 +1154,34 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>producer / loan officer</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>UFCU</t>
+          <t>Velocio Mortgage LLC</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Lyndee Bennett</t>
+          <t>Jerry Villarreal</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Manager, Brand &amp; Communications</t>
+          <t>residential mortgage LO (NMLS 1726390)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>lbennett@ufcu.org</t>
+          <t>GVgvillarreal@velociomortgage.com</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1191,39 +1191,39 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>512-467-8080</t>
+          <t>512-314-7301</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>local marketing</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>UFCU</t>
+          <t>Velocio Mortgage LLC</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Raquel Garcia</t>
+          <t>Brandon Burkhardt</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Marketing Director</t>
+          <t>residential mortgage LO (NMLS 917247)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>RGarcia@ufcu.org</t>
+          <t>BBurkhardt@velociomortgage.com</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1233,12 +1233,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>512-467-8080</t>
+          <t>512-314-7301</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>local marketing</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
@@ -1255,17 +1255,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Terrie Doggett</t>
+          <t>Lyndee Bennett</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Mortgage Services</t>
+          <t>Manager, Brand &amp; Communications</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>tdoggett@ufcu.org</t>
+          <t>lbennett@ufcu.org</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>producer / loan officer</t>
+          <t>local marketing</t>
         </is>
       </c>
     </row>
@@ -1297,13 +1297,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Shelly Martinez</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
+          <t>Raquel Garcia</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Marketing Director</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>smartinez@ufcu.org</t>
+          <t>RGarcia@ufcu.org</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1318,34 +1322,34 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>no title given</t>
+          <t>local marketing</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>First United Mortgage Group</t>
+          <t>UFCU</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Bryan Ezzell</t>
+          <t>Terrie Doggett</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>SVP/managing director</t>
+          <t>Mortgage Services</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>bryan.ezzell@firstunitedbank.com</t>
+          <t>tdoggett@ufcu.org</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1355,39 +1359,35 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>972-372-6800</t>
+          <t>512-467-8080</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>company exec (local-HQ shop)</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>LoanPeople</t>
+          <t>UFCU</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Max Leaman</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
+          <t>Shelly Martinez</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>max.leaman@loanpeople.com</t>
+          <t>smartinez@ufcu.org</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1397,39 +1397,39 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>512-886-4450</t>
+          <t>512-467-8080</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>company exec (local-HQ shop)</t>
+          <t>no title given</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>LoanPeople</t>
+          <t>First United Mortgage Group</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Dana Leaman</t>
+          <t>Bryan Ezzell</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>CMO</t>
+          <t>SVP/managing director</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Dana@maxleaman.com</t>
+          <t>bryan.ezzell@firstunitedbank.com</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>512-886-4450</t>
+          <t>972-372-6800</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1451,27 +1451,27 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>PrimeLending, a PlainsCapital Co.</t>
+          <t>LoanPeople</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Dawn Robinson</t>
+          <t>Max Leaman</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>SVP/Southwest regional manager</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>drobinson@primelending.com</t>
+          <t>max.leaman@loanpeople.com</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>512-381-4642</t>
+          <t>512-886-4450</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1493,69 +1493,69 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Pulte Mortgage LLC</t>
+          <t>LoanPeople</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pablo Rivas</t>
+          <t>Dana Leaman</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Division president</t>
+          <t>CMO</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>pablo.rivas@pultegroup.com</t>
+          <t>Dana@maxleaman.com</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>from your list</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>512-532-3347</t>
+          <t>512-886-4450</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
+          <t>company exec (local-HQ shop)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>KBHS Home Loans LLC</t>
+          <t>PrimeLending, a PlainsCapital Co.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Tanya Russell</t>
+          <t>Dawn Robinson</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Branch manager</t>
+          <t>SVP/Southwest regional manager</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>trussell1@kbhshomeloans.com</t>
+          <t>drobinson@primelending.com</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1565,39 +1565,39 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>855-378-6625</t>
+          <t>512-381-4642</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>company exec (local-HQ shop)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Cadence Bank</t>
+          <t>Pulte Mortgage LLC</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>David Grove</t>
+          <t>Pablo Rivas</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Austin division president</t>
+          <t>Division president</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>david.grove@cadencebank.com</t>
+          <t>pablo.rivas@pultegroup.com</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>512-231-8821</t>
+          <t>512-532-3347</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1619,27 +1619,27 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Cadence Bank</t>
+          <t>KBHS Home Loans LLC</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Aaron Dominguez</t>
+          <t>Tanya Russell</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>Branch manager</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>aaron.dominguez@bxs.com</t>
+          <t>trussell1@kbhshomeloans.com</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1649,12 +1649,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>512-231-8821</t>
+          <t>855-378-6625</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
@@ -1671,18 +1671,22 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Danielle Kernell</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
+          <t>David Grove</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Austin division president</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Danielle.Kernell@cadencebank.com</t>
+          <t>david.grove@cadencebank.com</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>from your list</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1692,7 +1696,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>no title given</t>
+          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
         </is>
       </c>
     </row>
@@ -1709,126 +1713,130 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
+          <t>Aaron Dominguez</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>aaron.dominguez@bxs.com</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>512-231-8821</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Cadence Bank</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Danielle Kernell</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Danielle.Kernell@cadencebank.com</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>512-231-8821</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>no title given</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Cadence Bank</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>Donald R. Grobowsky</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>donald.grobowsky@cadencebank.com</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>predicted (not verified)</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>512-231-8821</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>no title given | format 'first.last' confirmed at this domain, no credit</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>M/I Financial LLC</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Norm Lajewski</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Branch manager</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>no email found</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>512-770-8440</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>local market leader / branch decision-maker</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Bank of America Home Loans</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Cindy Chism</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>SVP-Austin home loans manager</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>no email found</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>512-691-0751</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Bank of America Home Loans</t>
+          <t>M/I Financial LLC</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>David Bader</t>
+          <t>Norm Lajewski</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Austin president</t>
+          <t>Branch manager</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -1839,96 +1847,88 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
+          <t>512-770-8440</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Bank of America Home Loans</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Cindy Chism</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>SVP-Austin home loans manager</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>no email found</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
           <t>512-691-0751</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Brightland Mortgage Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Rachel Shields</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>LO</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>rshields@BrightlandMortgage.com</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>from your list</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>512-365-4984</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>producer / loan officer</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Brightland Mortgage Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Evelyn Prince</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>residential mortgage LO</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>eprince@BrightlandMortgage.com</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>from your list</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>512-365-4984</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>producer / loan officer</t>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Bank of America Home Loans</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>David Bader</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Austin president</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>no email found</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>512-691-0751</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
@@ -1945,17 +1945,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Crystal Ramsey</t>
+          <t>Rachel Shields</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>sales manager</t>
+          <t>LO</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>cramsey@brightlandmortgage.com</t>
+          <t>rshields@BrightlandMortgage.com</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1970,34 +1970,34 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Guild Mortgage Company LLC</t>
+          <t>Brightland Mortgage Services Ltd.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Chad Overhauser</t>
+          <t>Evelyn Prince</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Divisional VP</t>
+          <t>residential mortgage LO</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>coverhauser@guildmortgage.net</t>
+          <t>eprince@BrightlandMortgage.com</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2007,39 +2007,39 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>512-335-5300</t>
+          <t>512-365-4984</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Guild Mortgage Company LLC</t>
+          <t>Brightland Mortgage Services Ltd.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Eric Weiss</t>
+          <t>Crystal Ramsey</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>RVP</t>
+          <t>sales manager</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>eweiss@guildmortgage.net</t>
+          <t>cramsey@brightlandmortgage.com</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2049,39 +2049,39 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>512-335-5300</t>
+          <t>512-365-4984</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Prosperity Bank</t>
+          <t>Guild Mortgage Company LLC</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Chip Bray</t>
+          <t>Chad Overhauser</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Area president</t>
+          <t>Divisional VP</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>chip.bray@prosperitybankusa.com</t>
+          <t>coverhauser@guildmortgage.net</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>512-472-5433</t>
+          <t>512-335-5300</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2103,27 +2103,27 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Prosperity Bank</t>
+          <t>Guild Mortgage Company LLC</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Brent Weber</t>
+          <t>Eric Weiss</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Area President</t>
+          <t>RVP</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>brent.weber@prosperitybankusa.com</t>
+          <t>eweiss@guildmortgage.net</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>512-472-5433</t>
+          <t>512-335-5300</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2155,17 +2155,17 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Eddie Safady</t>
+          <t>Chip Bray</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Vice chairman</t>
+          <t>Area president</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>eddie.safady@prosperitybankusa.com</t>
+          <t>chip.bray@prosperitybankusa.com</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2180,34 +2180,34 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>company exec (local-HQ shop)</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Morgan Stanley Private Bank NA</t>
+          <t>Prosperity Bank</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Jeremy L. Vance</t>
+          <t>Brent Weber</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>VP, private banker (Mortgage Co. list contact)</t>
+          <t>Area President</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>jeremy.vance@ms.com</t>
+          <t>brent.weber@prosperitybankusa.com</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2217,39 +2217,39 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>512-479-5707</t>
+          <t>512-472-5433</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Ark-la-tex Financial Services dba Benchmark</t>
+          <t>Prosperity Bank</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Tommy Nelms</t>
+          <t>Eddie Safady</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Senior branch manager</t>
+          <t>Vice chairman</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>tommy.nelms@benchmark.us</t>
+          <t>eddie.safady@prosperitybankusa.com</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2259,39 +2259,39 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>512-804-9393</t>
+          <t>512-472-5433</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>company exec (local-HQ shop)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Mission Mortgage of Texas Inc.</t>
+          <t>Morgan Stanley Private Bank NA</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Leigh Ann McCoy</t>
+          <t>Jeremy L. Vance</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>President</t>
+          <t>VP, private banker (Mortgage Co. list contact)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>lamccoy@missionmortgage.com</t>
+          <t>jeremy.vance@ms.com</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2301,115 +2301,123 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>512-328-0400</t>
+          <t>512-479-5707</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>company exec (local-HQ shop)</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Ark-la-tex Financial Services dba Benchmark</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Tommy Nelms</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Senior branch manager</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>tommy.nelms@benchmark.us</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>512-804-9393</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Mission Mortgage of Texas Inc.</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Lesley Guerrero</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Director of Mortgage Operations</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>lguerrero@missionmortgage.com</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>from your list</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Leigh Ann McCoy</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>lamccoy@missionmortgage.com</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>512-328-0400</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>Wells Fargo Bank NA</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Ben Murray</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>SVP/regional executive, branch banking</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>no email found</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr"/>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>local market leader / branch decision-maker</t>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>company exec (local-HQ shop)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Frost Bank</t>
+          <t>Mission Mortgage of Texas Inc.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Tim Crowley</t>
+          <t>Lesley Guerrero</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Austin region president</t>
+          <t>Director of Mortgage Operations</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>tcrowley@frostbank.com</t>
+          <t>lguerrero@missionmortgage.com</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2419,81 +2427,73 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>512-473-4343</t>
+          <t>512-328-0400</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
+          <t>other</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Wells Fargo Bank NA</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Ben Murray</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>SVP/regional executive, branch banking</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>no email found</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
           <t>local market leader / branch decision-maker</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Frost Bank</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Sallie Newman</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>VP marketing</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>snewman@frostbank.com</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>from your list</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>512-473-4343</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>local marketing</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Randolph-Brooks Federal Credit Union</t>
+          <t>Frost Bank</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Mark Sekula</t>
+          <t>Tim Crowley</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>President/CEO</t>
+          <t>Austin region president</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>msekula@rbfcu.org</t>
+          <t>tcrowley@frostbank.com</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2501,37 +2501,41 @@
           <t>from your list</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>512-473-4343</t>
+        </is>
+      </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>company exec (local-HQ shop)</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Roscoe Bank, a division of Cornerstone Capital Bank SSB</t>
+          <t>Frost Bank</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Rick Womble</t>
+          <t>Sallie Newman</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Market president</t>
+          <t>VP marketing</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>rwomble@roscoestatebank.com</t>
+          <t>snewman@frostbank.com</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2541,39 +2545,39 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>512-303-1800</t>
+          <t>512-473-4343</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>local marketing</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Roscoe Bank, a division of Cornerstone Capital Bank SSB</t>
+          <t>Randolph-Brooks Federal Credit Union</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>John Lovelance</t>
+          <t>Mark Sekula</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>AVP</t>
+          <t>President/CEO</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>jlovelace@roscoebank.com</t>
+          <t>msekula@rbfcu.org</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2581,83 +2585,79 @@
           <t>from your list</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>512-303-1800</t>
-        </is>
-      </c>
+      <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>company exec (local-HQ shop)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Southern Lending Services</t>
+          <t>Roscoe Bank, a division of Cornerstone Capital Bank SSB</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>William Dorgan</t>
+          <t>Rick Womble</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>SVP/Production manager</t>
+          <t>Market president</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>wdorgan@southernlendingservices.com</t>
+          <t>rwomble@roscoestatebank.com</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>found by pattern test</t>
+          <t>from your list</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>512-617-3067</t>
+          <t>512-303-1800</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker | NeverBounce pattern test, no Apollo credit</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Movement Mortgage</t>
+          <t>Roscoe Bank, a division of Cornerstone Capital Bank SSB</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Dan Reagan</t>
+          <t>John Lovelance</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Market Leader</t>
+          <t>AVP</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>dan.reagan@movement.com</t>
+          <t>jlovelace@roscoebank.com</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2667,54 +2667,54 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>512-947-1700</t>
+          <t>512-303-1800</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>56</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Movement Mortgage</t>
+          <t>Southern Lending Services</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Bobby Shull</t>
+          <t>William Dorgan</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Market leader</t>
+          <t>SVP/Production manager</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>bobby.shull@movement.com</t>
+          <t>wdorgan@southernlendingservices.com</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>from your list</t>
+          <t>found by pattern test</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>512-947-1700</t>
+          <t>512-617-3067</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>local market leader / branch decision-maker | NeverBounce pattern test, no Apollo credit</t>
         </is>
       </c>
     </row>
@@ -2731,17 +2731,17 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Michael Task</t>
+          <t>Dan Reagan</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Loan originator</t>
+          <t>Market Leader</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>michael.task@movement.com</t>
+          <t>dan.reagan@movement.com</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>producer / loan officer</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
@@ -2773,13 +2773,17 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Trish Busch</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr"/>
+          <t>Bobby Shull</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Market leader</t>
+        </is>
+      </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>trish.busch@movement.com</t>
+          <t>bobby.shull@movement.com</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2794,72 +2798,72 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>no title given</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>57</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>UBS Bank USA</t>
+          <t>Movement Mortgage</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Jeff Bidstrup</t>
+          <t>Michael Task</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Market director</t>
+          <t>Loan originator</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>jeff.bidstrup@ubs.com</t>
+          <t>michael.task@movement.com</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>512-947-1700</t>
+        </is>
+      </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
+          <t>producer / loan officer</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>57</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Truist Bank</t>
+          <t>Movement Mortgage</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Stephen Smith</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Market president</t>
-        </is>
-      </c>
+          <t>Trish Busch</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr"/>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>SMSmith@truist.com</t>
+          <t>trish.busch@movement.com</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2869,207 +2873,203 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>512-472-7770</t>
+          <t>512-947-1700</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>no title given</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>62</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Truist Bank</t>
+          <t>UBS Bank USA</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Cindy Montgomery</t>
+          <t>Jeff Bidstrup</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Retail/Communications</t>
+          <t>Market director</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Cynthia.Montgomery@truist.com</t>
+          <t>jeff.bidstrup@ubs.com</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>from your list</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>512-472-7770</t>
-        </is>
-      </c>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>64</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Charles Schwab Bank, SSB</t>
+          <t>Truist Bank</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Richard Brandi</t>
+          <t>Stephen Smith</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>VP/Branch manager</t>
+          <t>Market president</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>richard.brandi@schwab.com</t>
+          <t>SMSmith@truist.com</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>from your list</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>512-370-3880</t>
+          <t>512-472-7770</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>64</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>SWBC</t>
+          <t>Truist Bank</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Charlie Amato</t>
+          <t>Cindy Montgomery</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>co-top local exec</t>
+          <t>Retail/Communications</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>camato@swbc.com</t>
+          <t>Cynthia.Montgomery@truist.com</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>found by pattern test</t>
+          <t>from your list</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>210-525-1241</t>
+          <t>512-472-7770</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>other | NeverBounce pattern test, no Apollo credit</t>
+          <t>other</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>66</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>SWBC</t>
+          <t>Charles Schwab Bank, SSB</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Gary Dudley</t>
+          <t>Richard Brandi</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>co-top local exec</t>
+          <t>VP/Branch manager</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>gdudley@swbc.com</t>
+          <t>richard.brandi@schwab.com</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>found by pattern test</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>210-525-1241</t>
+          <t>512-370-3880</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>other | NeverBounce pattern test, no Apollo credit</t>
+          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>70</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Southstate Bank, National Association</t>
+          <t>SWBC</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Hunter Adams</t>
+          <t>Charlie Amato</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Branch manager</t>
+          <t>co-top local exec</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>hunter.adams@southstatebank.com</t>
+          <t>camato@swbc.com</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3079,165 +3079,165 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>512-652-0404</t>
+          <t>210-525-1241</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker | NeverBounce pattern test, no Apollo credit</t>
+          <t>other | NeverBounce pattern test, no Apollo credit</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>70</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Southstate Bank, National Association</t>
+          <t>SWBC</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>John Corbett</t>
+          <t>Gary Dudley</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>co-top local exec</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>jcorbett@southstatebank.com</t>
+          <t>gdudley@swbc.com</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>found by pattern test</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>512-652-0404</t>
+          <t>210-525-1241</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>company exec (local-HQ shop) | apollo (credit spent)</t>
+          <t>other | NeverBounce pattern test, no Apollo credit</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>72</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>SouthStar Bank SSB</t>
+          <t>Southstate Bank, National Association</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Brent Gibbs</t>
+          <t>Hunter Adams</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>EVP/Central Texas president</t>
+          <t>Branch manager</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>brent.gibbs@southstarbank.com</t>
+          <t>hunter.adams@southstatebank.com</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>from your list</t>
+          <t>found by pattern test</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>512-288-3322</t>
+          <t>512-652-0404</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>local market leader / branch decision-maker | NeverBounce pattern test, no Apollo credit</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>72</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>SouthStar Bank SSB</t>
+          <t>Southstate Bank, National Association</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Keely McCarthy</t>
+          <t>John Corbett</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Vice President of Marketing</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>keely.mccarthy@southstarbank.com</t>
+          <t>jcorbett@southstatebank.com</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>from your list</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>512-288-3322</t>
+          <t>512-652-0404</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>local marketing</t>
+          <t>company exec (local-HQ shop) | apollo (credit spent)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>75</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Lower</t>
+          <t>SouthStar Bank SSB</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Stacey Smith</t>
+          <t>Brent Gibbs</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Branch manager</t>
+          <t>EVP/Central Texas president</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>stacey.smith@lower.com</t>
+          <t>brent.gibbs@southstarbank.com</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>512-750-4320</t>
+          <t>512-288-3322</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3259,103 +3259,111 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>75</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Amplify Credit Union</t>
+          <t>SouthStar Bank SSB</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Kendall Garrison</t>
+          <t>Keely McCarthy</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>CEO/president</t>
+          <t>Vice President of Marketing</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>kgarrison@goamplify.com</t>
+          <t>keely.mccarthy@southstarbank.com</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>from your list</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>512-836-5901</t>
+          <t>512-288-3322</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>company exec (local-HQ shop) | apollo (credit spent)</t>
+          <t>local marketing</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>BOK Financial Mortgage</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>Corey Enlow</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr"/>
-      <c r="E70" s="3" t="inlineStr"/>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>no email found</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>844-517-3308</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>no title given</t>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Lower</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Stacey Smith</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Branch manager</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>stacey.smith@lower.com</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>512-750-4320</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Encompass Lending Group</t>
+          <t>Amplify Credit Union</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Josh Bibler</t>
+          <t>Kendall Garrison</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Regional VP</t>
+          <t>CEO/president</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>jbibler@encompasslending.com</t>
+          <t>kgarrison@goamplify.com</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3365,138 +3373,130 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>512-587-9500</t>
+          <t>512-836-5901</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
+          <t>company exec (local-HQ shop) | apollo (credit spent)</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>93</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>Residential Wholesale Mortgage</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Steve Ferguson</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>Branch manager</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>steve@rwmloans.com</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>512-913-7566</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>BOK Financial Mortgage</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Corey Enlow</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr"/>
+      <c r="E72" s="3" t="inlineStr"/>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>no email found</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>844-517-3308</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>no title given</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>90</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Security State Bank &amp; Trust</t>
+          <t>Encompass Lending Group</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Tim Craig</t>
+          <t>Josh Bibler</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Branch President, Liberty Hill</t>
+          <t>Regional VP</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>tcraig@ssbtexas.com</t>
+          <t>jbibler@encompasslending.com</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>from your list</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>512-263-1600</t>
+          <t>512-587-9500</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>93</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Security State Bank &amp; Trust</t>
+          <t>Residential Wholesale Mortgage</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Brian Thibodeaux</t>
+          <t>Steve Ferguson</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Branch president, Dripping Springs</t>
+          <t>Branch manager</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>bthibodeaux@ssbtexas.com</t>
+          <t>steve@rwmloans.com</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>from your list</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>512-263-1600</t>
+          <t>512-913-7566</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>local market leader / branch decision-maker</t>
+          <t>local market leader / branch decision-maker | apollo (credit spent)</t>
         </is>
       </c>
     </row>
@@ -3513,17 +3513,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Donna Hensley</t>
+          <t>Tim Craig</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Branch president, Lago Vista</t>
+          <t>Branch President, Liberty Hill</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>dhensley@ssbtexas.com</t>
+          <t>tcraig@ssbtexas.com</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3555,17 +3555,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Joe David Sherrod</t>
+          <t>Brian Thibodeaux</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Branch president, Spicewood (Paleface, Bee Cave)</t>
+          <t>Branch president, Dripping Springs</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>jsherrod@ssbtexas.com</t>
+          <t>bthibodeaux@ssbtexas.com</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3587,47 +3587,131 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Security State Bank &amp; Trust</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Donna Hensley</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Branch president, Lago Vista</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>dhensley@ssbtexas.com</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>512-263-1600</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Security State Bank &amp; Trust</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Joe David Sherrod</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Branch president, Spicewood (Paleface, Bee Cave)</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>jsherrod@ssbtexas.com</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>from your list</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>512-263-1600</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>local market leader / branch decision-maker</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
           <t>99</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>Canopy Mortgage</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>E. Lee Smith</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>Branch manager</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>esmith@canopymortgage.com</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>found by pattern test</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>512-598-9093</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>local market leader / branch decision-maker | NeverBounce pattern test, no Apollo credit</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H77"/>
+  <autoFilter ref="A1:H79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3638,14 +3722,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3666,11 +3749,6 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
           <t>Phone</t>
         </is>
       </c>
@@ -3678,81 +3756,66 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>DHI Mortgage Co. Ltd.</t>
+          <t>Fairway Independent Mortgage Corp. - Round Rock</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Eddie Garza De Haro</t>
+          <t>Steve Jacobson</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>branch sales manager</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>dhimortgage.com</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>512-502-0545</t>
+          <t>512-776-1420</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Fairway Independent Mortgage Corp. - Round Rock</t>
+          <t>M/I Financial LLC</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Steve Jacobson</t>
+          <t>Norm Lajewski</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Branch manager</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>fairway.com</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>512-776-1420</t>
+          <t>512-770-8440</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>M/I Financial LLC</t>
+          <t>Bank of America Home Loans</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Norm Lajewski</t>
+          <t>Cindy Chism</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Branch manager</t>
+          <t>SVP-Austin home loans manager</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>mihomes.com</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>512-770-8440</t>
+          <t>512-691-0751</t>
         </is>
       </c>
     </row>
@@ -3764,20 +3827,15 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Cindy Chism</t>
+          <t>David Bader</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>SVP-Austin home loans manager</t>
+          <t>Austin president</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>bankofamerica.com</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>512-691-0751</t>
         </is>
@@ -3786,139 +3844,36 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Bank of America Home Loans</t>
+          <t>Wells Fargo Bank NA</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>David Bader</t>
+          <t>Ben Murray</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Austin president</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>bankofamerica.com</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>512-691-0751</t>
-        </is>
-      </c>
+          <t>SVP/regional executive, branch banking</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Wells Fargo Bank NA</t>
+          <t>BOK Financial Mortgage</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ben Murray</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>SVP/regional executive, branch banking</t>
-        </is>
-      </c>
+          <t>Corey Enlow</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>wellsfargo.com</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>BOK Financial Mortgage</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Corey Enlow</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>bokfinancial.com</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
           <t>844-517-3308</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="118" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>122 contacts in, 76 kept across 41 companies. 69 now have an email; 7 still do not.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>8 Apollo credits and 85 NeverBounce credits spent. Apollo balance untouched otherwise; NeverBounce is at 710.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Loan officers were kept on purpose. Residential LOs are commission-based and buy their own marketing, so a producer can be a better prospect than their branch manager - the opposite of how I treated bank VPs and accounting-firm Directors on your other lists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Rows marked 'predicted (not verified)' were built from a format confirmed elsewhere at that company. Donald Grobowsky at Cadence is the only one - David Grove's verified address confirmed the first.last pattern.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Rows found by 'NeverBounce pattern test' were guessed and then confirmed to be live mailboxes. Treat them as real but not Apollo-verified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>The 8 still missing are mostly at very large banks (Bank of America, Wells Fargo, BOK) where Apollo has no record under that name. Their phone numbers are in your list - these are call-first targets, not email targets.</t>
         </is>
       </c>
     </row>

</xml_diff>